<commit_message>
some ui fixes, updated excel
</commit_message>
<xml_diff>
--- a/question/game_ques.xlsx
+++ b/question/game_ques.xlsx
@@ -2806,9 +2806,8 @@
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="15.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="15.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
@@ -2844,10 +2843,10 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="0" t="s">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
@@ -2882,7 +2881,7 @@
       <c r="J2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M2" s="3" t="n">
@@ -2917,7 +2916,7 @@
       <c r="J3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2949,7 +2948,7 @@
       <c r="J4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="K4" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2981,7 +2980,7 @@
       <c r="J5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="K5" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3013,7 +3012,7 @@
       <c r="J6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K6" s="0" t="s">
+      <c r="K6" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3045,7 +3044,7 @@
       <c r="J7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K7" s="0" t="s">
+      <c r="K7" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3077,7 +3076,7 @@
       <c r="J8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="0" t="s">
+      <c r="K8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3109,7 +3108,7 @@
       <c r="J9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="0" t="s">
+      <c r="K9" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3141,7 +3140,7 @@
       <c r="J10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K10" s="0" t="s">
+      <c r="K10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3173,7 +3172,7 @@
       <c r="J11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K11" s="0" t="s">
+      <c r="K11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3205,10 +3204,10 @@
       <c r="J12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="0" t="s">
+      <c r="K12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L12" s="0" t="s">
+      <c r="L12" s="1" t="s">
         <v>18</v>
       </c>
       <c r="M12" s="3" t="n">
@@ -3243,10 +3242,10 @@
       <c r="J13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="0" t="s">
+      <c r="K13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L13" s="0" t="s">
+      <c r="L13" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3278,10 +3277,10 @@
       <c r="J14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="0" t="s">
+      <c r="K14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L14" s="0" t="s">
+      <c r="L14" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3313,10 +3312,10 @@
       <c r="J15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="0" t="s">
+      <c r="K15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L15" s="0" t="s">
+      <c r="L15" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3348,10 +3347,10 @@
       <c r="J16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="0" t="s">
+      <c r="K16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L16" s="0" t="s">
+      <c r="L16" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3383,10 +3382,10 @@
       <c r="J17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="0" t="s">
+      <c r="K17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L17" s="0" t="s">
+      <c r="L17" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3418,10 +3417,10 @@
       <c r="J18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="0" t="s">
+      <c r="K18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L18" s="0" t="s">
+      <c r="L18" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3453,10 +3452,10 @@
       <c r="J19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K19" s="0" t="s">
+      <c r="K19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L19" s="0" t="s">
+      <c r="L19" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3488,10 +3487,10 @@
       <c r="J20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K20" s="0" t="s">
+      <c r="K20" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L20" s="0" t="s">
+      <c r="L20" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3523,10 +3522,10 @@
       <c r="J21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="0" t="s">
+      <c r="K21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L21" s="0" t="s">
+      <c r="L21" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3558,10 +3557,10 @@
       <c r="J22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K22" s="0" t="s">
+      <c r="K22" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L22" s="0" t="s">
+      <c r="L22" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M22" s="3" t="n">
@@ -3596,10 +3595,10 @@
       <c r="J23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K23" s="0" t="s">
+      <c r="K23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L23" s="0" t="s">
+      <c r="L23" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3631,10 +3630,10 @@
       <c r="J24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K24" s="0" t="s">
+      <c r="K24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L24" s="0" t="s">
+      <c r="L24" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3666,10 +3665,10 @@
       <c r="J25" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K25" s="0" t="s">
+      <c r="K25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L25" s="0" t="s">
+      <c r="L25" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3701,10 +3700,10 @@
       <c r="J26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K26" s="0" t="s">
+      <c r="K26" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L26" s="0" t="s">
+      <c r="L26" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3736,10 +3735,10 @@
       <c r="J27" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K27" s="0" t="s">
+      <c r="K27" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L27" s="0" t="s">
+      <c r="L27" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3771,10 +3770,10 @@
       <c r="J28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K28" s="0" t="s">
+      <c r="K28" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L28" s="0" t="s">
+      <c r="L28" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3806,10 +3805,10 @@
       <c r="J29" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K29" s="0" t="s">
+      <c r="K29" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L29" s="0" t="s">
+      <c r="L29" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3841,10 +3840,10 @@
       <c r="J30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K30" s="0" t="s">
+      <c r="K30" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L30" s="0" t="s">
+      <c r="L30" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3876,10 +3875,10 @@
       <c r="J31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K31" s="0" t="s">
+      <c r="K31" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L31" s="0" t="s">
+      <c r="L31" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -3911,10 +3910,10 @@
       <c r="J32" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K32" s="0" t="s">
+      <c r="K32" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L32" s="0" t="s">
+      <c r="L32" s="1" t="s">
         <v>32</v>
       </c>
       <c r="M32" s="3" t="n">
@@ -3949,10 +3948,10 @@
       <c r="J33" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K33" s="0" t="s">
+      <c r="K33" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L33" s="0" t="s">
+      <c r="L33" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3984,10 +3983,10 @@
       <c r="J34" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K34" s="0" t="s">
+      <c r="K34" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L34" s="0" t="s">
+      <c r="L34" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4019,10 +4018,10 @@
       <c r="J35" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K35" s="0" t="s">
+      <c r="K35" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L35" s="0" t="s">
+      <c r="L35" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4054,10 +4053,10 @@
       <c r="J36" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K36" s="0" t="s">
+      <c r="K36" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L36" s="0" t="s">
+      <c r="L36" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4089,10 +4088,10 @@
       <c r="J37" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K37" s="0" t="s">
+      <c r="K37" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L37" s="0" t="s">
+      <c r="L37" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4124,10 +4123,10 @@
       <c r="J38" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K38" s="0" t="s">
+      <c r="K38" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L38" s="0" t="s">
+      <c r="L38" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4159,10 +4158,10 @@
       <c r="J39" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K39" s="0" t="s">
+      <c r="K39" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L39" s="0" t="s">
+      <c r="L39" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4194,10 +4193,10 @@
       <c r="J40" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K40" s="0" t="s">
+      <c r="K40" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L40" s="0" t="s">
+      <c r="L40" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4229,10 +4228,10 @@
       <c r="J41" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K41" s="0" t="s">
+      <c r="K41" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L41" s="0" t="s">
+      <c r="L41" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4264,10 +4263,10 @@
       <c r="J42" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K42" s="0" t="s">
+      <c r="K42" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L42" s="0" t="s">
+      <c r="L42" s="1" t="s">
         <v>46</v>
       </c>
       <c r="M42" s="3" t="n">
@@ -4302,10 +4301,10 @@
       <c r="J43" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K43" s="0" t="s">
+      <c r="K43" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L43" s="0" t="s">
+      <c r="L43" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4337,10 +4336,10 @@
       <c r="J44" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K44" s="0" t="s">
+      <c r="K44" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L44" s="0" t="s">
+      <c r="L44" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4372,10 +4371,10 @@
       <c r="J45" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K45" s="0" t="s">
+      <c r="K45" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L45" s="0" t="s">
+      <c r="L45" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4407,10 +4406,10 @@
       <c r="J46" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K46" s="0" t="s">
+      <c r="K46" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L46" s="0" t="s">
+      <c r="L46" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4442,10 +4441,10 @@
       <c r="J47" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K47" s="0" t="s">
+      <c r="K47" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L47" s="0" t="s">
+      <c r="L47" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4477,10 +4476,10 @@
       <c r="J48" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K48" s="0" t="s">
+      <c r="K48" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L48" s="0" t="s">
+      <c r="L48" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4512,10 +4511,10 @@
       <c r="J49" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K49" s="0" t="s">
+      <c r="K49" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L49" s="0" t="s">
+      <c r="L49" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4547,10 +4546,10 @@
       <c r="J50" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K50" s="0" t="s">
+      <c r="K50" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L50" s="0" t="s">
+      <c r="L50" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4582,10 +4581,10 @@
       <c r="J51" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K51" s="0" t="s">
+      <c r="K51" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="L51" s="0" t="s">
+      <c r="L51" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -4617,10 +4616,10 @@
       <c r="J52" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K52" s="0" t="s">
+      <c r="K52" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L52" s="0" t="s">
+      <c r="L52" s="1" t="s">
         <v>60</v>
       </c>
       <c r="M52" s="3" t="n">
@@ -4655,10 +4654,10 @@
       <c r="J53" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K53" s="0" t="s">
+      <c r="K53" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L53" s="0" t="s">
+      <c r="L53" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4690,10 +4689,10 @@
       <c r="J54" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K54" s="0" t="s">
+      <c r="K54" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L54" s="0" t="s">
+      <c r="L54" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4725,10 +4724,10 @@
       <c r="J55" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K55" s="0" t="s">
+      <c r="K55" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L55" s="0" t="s">
+      <c r="L55" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4760,10 +4759,10 @@
       <c r="J56" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K56" s="0" t="s">
+      <c r="K56" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L56" s="0" t="s">
+      <c r="L56" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4795,10 +4794,10 @@
       <c r="J57" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K57" s="0" t="s">
+      <c r="K57" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L57" s="0" t="s">
+      <c r="L57" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4830,10 +4829,10 @@
       <c r="J58" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K58" s="0" t="s">
+      <c r="K58" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L58" s="0" t="s">
+      <c r="L58" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4865,10 +4864,10 @@
       <c r="J59" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K59" s="0" t="s">
+      <c r="K59" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L59" s="0" t="s">
+      <c r="L59" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4900,10 +4899,10 @@
       <c r="J60" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K60" s="0" t="s">
+      <c r="K60" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L60" s="0" t="s">
+      <c r="L60" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4935,10 +4934,10 @@
       <c r="J61" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="K61" s="0" t="s">
+      <c r="K61" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L61" s="0" t="s">
+      <c r="L61" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -4970,10 +4969,10 @@
       <c r="J62" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K62" s="0" t="s">
+      <c r="K62" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L62" s="0" t="s">
+      <c r="L62" s="1" t="s">
         <v>70</v>
       </c>
       <c r="M62" s="3" t="n">
@@ -5008,10 +5007,10 @@
       <c r="J63" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K63" s="0" t="s">
+      <c r="K63" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L63" s="0" t="s">
+      <c r="L63" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5043,10 +5042,10 @@
       <c r="J64" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K64" s="0" t="s">
+      <c r="K64" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L64" s="0" t="s">
+      <c r="L64" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5078,10 +5077,10 @@
       <c r="J65" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K65" s="0" t="s">
+      <c r="K65" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L65" s="0" t="s">
+      <c r="L65" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5113,10 +5112,10 @@
       <c r="J66" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K66" s="0" t="s">
+      <c r="K66" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L66" s="0" t="s">
+      <c r="L66" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5148,10 +5147,10 @@
       <c r="J67" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K67" s="0" t="s">
+      <c r="K67" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L67" s="0" t="s">
+      <c r="L67" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5183,10 +5182,10 @@
       <c r="J68" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K68" s="0" t="s">
+      <c r="K68" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L68" s="0" t="s">
+      <c r="L68" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5218,10 +5217,10 @@
       <c r="J69" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K69" s="0" t="s">
+      <c r="K69" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L69" s="0" t="s">
+      <c r="L69" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5253,10 +5252,10 @@
       <c r="J70" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K70" s="0" t="s">
+      <c r="K70" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L70" s="0" t="s">
+      <c r="L70" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5288,10 +5287,10 @@
       <c r="J71" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="K71" s="0" t="s">
+      <c r="K71" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L71" s="0" t="s">
+      <c r="L71" s="1" t="s">
         <v>70</v>
       </c>
     </row>
@@ -5323,10 +5322,10 @@
       <c r="J72" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K72" s="0" t="s">
+      <c r="K72" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L72" s="0" t="s">
+      <c r="L72" s="1" t="s">
         <v>81</v>
       </c>
       <c r="M72" s="3" t="n">
@@ -5361,10 +5360,10 @@
       <c r="J73" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K73" s="0" t="s">
+      <c r="K73" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L73" s="0" t="s">
+      <c r="L73" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5396,10 +5395,10 @@
       <c r="J74" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K74" s="0" t="s">
+      <c r="K74" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L74" s="0" t="s">
+      <c r="L74" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5431,10 +5430,10 @@
       <c r="J75" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K75" s="0" t="s">
+      <c r="K75" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L75" s="0" t="s">
+      <c r="L75" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5466,10 +5465,10 @@
       <c r="J76" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K76" s="0" t="s">
+      <c r="K76" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L76" s="0" t="s">
+      <c r="L76" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5501,10 +5500,10 @@
       <c r="J77" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K77" s="0" t="s">
+      <c r="K77" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L77" s="0" t="s">
+      <c r="L77" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5536,10 +5535,10 @@
       <c r="J78" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K78" s="0" t="s">
+      <c r="K78" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L78" s="0" t="s">
+      <c r="L78" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5571,10 +5570,10 @@
       <c r="J79" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K79" s="0" t="s">
+      <c r="K79" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L79" s="0" t="s">
+      <c r="L79" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5606,10 +5605,10 @@
       <c r="J80" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K80" s="0" t="s">
+      <c r="K80" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L80" s="0" t="s">
+      <c r="L80" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5641,10 +5640,10 @@
       <c r="J81" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="K81" s="0" t="s">
+      <c r="K81" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L81" s="0" t="s">
+      <c r="L81" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -5676,10 +5675,10 @@
       <c r="J82" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K82" s="0" t="s">
+      <c r="K82" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L82" s="0" t="s">
+      <c r="L82" s="1" t="s">
         <v>92</v>
       </c>
       <c r="M82" s="3" t="n">
@@ -5714,10 +5713,10 @@
       <c r="J83" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K83" s="0" t="s">
+      <c r="K83" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L83" s="0" t="s">
+      <c r="L83" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5749,10 +5748,10 @@
       <c r="J84" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K84" s="0" t="s">
+      <c r="K84" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L84" s="0" t="s">
+      <c r="L84" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5784,10 +5783,10 @@
       <c r="J85" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K85" s="0" t="s">
+      <c r="K85" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L85" s="0" t="s">
+      <c r="L85" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5819,10 +5818,10 @@
       <c r="J86" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K86" s="0" t="s">
+      <c r="K86" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L86" s="0" t="s">
+      <c r="L86" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5854,10 +5853,10 @@
       <c r="J87" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K87" s="0" t="s">
+      <c r="K87" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L87" s="0" t="s">
+      <c r="L87" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5889,10 +5888,10 @@
       <c r="J88" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K88" s="0" t="s">
+      <c r="K88" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L88" s="0" t="s">
+      <c r="L88" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5924,10 +5923,10 @@
       <c r="J89" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K89" s="0" t="s">
+      <c r="K89" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L89" s="0" t="s">
+      <c r="L89" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5959,10 +5958,10 @@
       <c r="J90" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K90" s="0" t="s">
+      <c r="K90" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L90" s="0" t="s">
+      <c r="L90" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -5994,10 +5993,10 @@
       <c r="J91" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K91" s="0" t="s">
+      <c r="K91" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L91" s="0" t="s">
+      <c r="L91" s="1" t="s">
         <v>92</v>
       </c>
     </row>
@@ -6029,10 +6028,10 @@
       <c r="J92" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K92" s="0" t="s">
+      <c r="K92" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L92" s="0" t="s">
+      <c r="L92" s="1" t="s">
         <v>104</v>
       </c>
       <c r="M92" s="3" t="n">
@@ -6067,10 +6066,10 @@
       <c r="J93" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K93" s="0" t="s">
+      <c r="K93" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L93" s="0" t="s">
+      <c r="L93" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6102,10 +6101,10 @@
       <c r="J94" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K94" s="0" t="s">
+      <c r="K94" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L94" s="0" t="s">
+      <c r="L94" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6137,10 +6136,10 @@
       <c r="J95" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K95" s="0" t="s">
+      <c r="K95" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L95" s="0" t="s">
+      <c r="L95" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6172,10 +6171,10 @@
       <c r="J96" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K96" s="0" t="s">
+      <c r="K96" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L96" s="0" t="s">
+      <c r="L96" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6207,10 +6206,10 @@
       <c r="J97" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K97" s="0" t="s">
+      <c r="K97" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L97" s="0" t="s">
+      <c r="L97" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6242,10 +6241,10 @@
       <c r="J98" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K98" s="0" t="s">
+      <c r="K98" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L98" s="0" t="s">
+      <c r="L98" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6277,10 +6276,10 @@
       <c r="J99" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K99" s="0" t="s">
+      <c r="K99" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L99" s="0" t="s">
+      <c r="L99" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6312,10 +6311,10 @@
       <c r="J100" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K100" s="0" t="s">
+      <c r="K100" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L100" s="0" t="s">
+      <c r="L100" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6347,10 +6346,10 @@
       <c r="J101" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K101" s="0" t="s">
+      <c r="K101" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="L101" s="0" t="s">
+      <c r="L101" s="1" t="s">
         <v>104</v>
       </c>
     </row>
@@ -6382,10 +6381,10 @@
       <c r="J102" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K102" s="0" t="s">
+      <c r="K102" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L102" s="0" t="s">
+      <c r="L102" s="1" t="s">
         <v>116</v>
       </c>
       <c r="M102" s="3" t="n">
@@ -6420,10 +6419,10 @@
       <c r="J103" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K103" s="0" t="s">
+      <c r="K103" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L103" s="0" t="s">
+      <c r="L103" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6455,10 +6454,10 @@
       <c r="J104" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K104" s="0" t="s">
+      <c r="K104" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L104" s="0" t="s">
+      <c r="L104" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6490,10 +6489,10 @@
       <c r="J105" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K105" s="0" t="s">
+      <c r="K105" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L105" s="0" t="s">
+      <c r="L105" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6525,10 +6524,10 @@
       <c r="J106" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K106" s="0" t="s">
+      <c r="K106" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L106" s="0" t="s">
+      <c r="L106" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6560,10 +6559,10 @@
       <c r="J107" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K107" s="0" t="s">
+      <c r="K107" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L107" s="0" t="s">
+      <c r="L107" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6595,10 +6594,10 @@
       <c r="J108" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K108" s="0" t="s">
+      <c r="K108" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L108" s="0" t="s">
+      <c r="L108" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6630,10 +6629,10 @@
       <c r="J109" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K109" s="0" t="s">
+      <c r="K109" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L109" s="0" t="s">
+      <c r="L109" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6665,10 +6664,10 @@
       <c r="J110" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K110" s="0" t="s">
+      <c r="K110" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L110" s="0" t="s">
+      <c r="L110" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6700,10 +6699,10 @@
       <c r="J111" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K111" s="0" t="s">
+      <c r="K111" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L111" s="0" t="s">
+      <c r="L111" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -6735,10 +6734,10 @@
       <c r="J112" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K112" s="0" t="s">
+      <c r="K112" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L112" s="0" t="s">
+      <c r="L112" s="1" t="s">
         <v>127</v>
       </c>
       <c r="M112" s="3" t="n">
@@ -6773,10 +6772,10 @@
       <c r="J113" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K113" s="0" t="s">
+      <c r="K113" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L113" s="0" t="s">
+      <c r="L113" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6808,10 +6807,10 @@
       <c r="J114" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K114" s="0" t="s">
+      <c r="K114" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L114" s="0" t="s">
+      <c r="L114" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6843,10 +6842,10 @@
       <c r="J115" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K115" s="0" t="s">
+      <c r="K115" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L115" s="0" t="s">
+      <c r="L115" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6878,10 +6877,10 @@
       <c r="J116" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K116" s="0" t="s">
+      <c r="K116" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L116" s="0" t="s">
+      <c r="L116" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6913,10 +6912,10 @@
       <c r="J117" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K117" s="0" t="s">
+      <c r="K117" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L117" s="0" t="s">
+      <c r="L117" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6948,10 +6947,10 @@
       <c r="J118" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K118" s="0" t="s">
+      <c r="K118" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L118" s="0" t="s">
+      <c r="L118" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -6983,10 +6982,10 @@
       <c r="J119" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K119" s="0" t="s">
+      <c r="K119" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L119" s="0" t="s">
+      <c r="L119" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -7018,10 +7017,10 @@
       <c r="J120" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K120" s="0" t="s">
+      <c r="K120" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L120" s="0" t="s">
+      <c r="L120" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -7053,10 +7052,10 @@
       <c r="J121" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K121" s="0" t="s">
+      <c r="K121" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="L121" s="0" t="s">
+      <c r="L121" s="1" t="s">
         <v>127</v>
       </c>
     </row>
@@ -7088,10 +7087,10 @@
       <c r="J122" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K122" s="0" t="s">
+      <c r="K122" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L122" s="0" t="s">
+      <c r="L122" s="1" t="s">
         <v>138</v>
       </c>
       <c r="M122" s="1" t="n">
@@ -7126,10 +7125,10 @@
       <c r="J123" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K123" s="0" t="s">
+      <c r="K123" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L123" s="0" t="s">
+      <c r="L123" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7161,10 +7160,10 @@
       <c r="J124" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K124" s="0" t="s">
+      <c r="K124" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L124" s="0" t="s">
+      <c r="L124" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7196,10 +7195,10 @@
       <c r="J125" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K125" s="0" t="s">
+      <c r="K125" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L125" s="0" t="s">
+      <c r="L125" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7231,10 +7230,10 @@
       <c r="J126" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K126" s="0" t="s">
+      <c r="K126" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L126" s="0" t="s">
+      <c r="L126" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7266,10 +7265,10 @@
       <c r="J127" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K127" s="0" t="s">
+      <c r="K127" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L127" s="0" t="s">
+      <c r="L127" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7301,10 +7300,10 @@
       <c r="J128" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K128" s="0" t="s">
+      <c r="K128" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L128" s="0" t="s">
+      <c r="L128" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7336,10 +7335,10 @@
       <c r="J129" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K129" s="0" t="s">
+      <c r="K129" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L129" s="0" t="s">
+      <c r="L129" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7371,10 +7370,10 @@
       <c r="J130" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K130" s="0" t="s">
+      <c r="K130" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L130" s="0" t="s">
+      <c r="L130" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7406,10 +7405,10 @@
       <c r="J131" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K131" s="0" t="s">
+      <c r="K131" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L131" s="0" t="s">
+      <c r="L131" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -7441,10 +7440,10 @@
       <c r="J132" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K132" s="0" t="s">
+      <c r="K132" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L132" s="0" t="s">
+      <c r="L132" s="1" t="s">
         <v>150</v>
       </c>
       <c r="M132" s="1" t="n">
@@ -7479,10 +7478,10 @@
       <c r="J133" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K133" s="0" t="s">
+      <c r="K133" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L133" s="0" t="s">
+      <c r="L133" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7514,10 +7513,10 @@
       <c r="J134" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K134" s="0" t="s">
+      <c r="K134" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L134" s="0" t="s">
+      <c r="L134" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7549,10 +7548,10 @@
       <c r="J135" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K135" s="0" t="s">
+      <c r="K135" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L135" s="0" t="s">
+      <c r="L135" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7584,10 +7583,10 @@
       <c r="J136" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K136" s="0" t="s">
+      <c r="K136" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L136" s="0" t="s">
+      <c r="L136" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7619,10 +7618,10 @@
       <c r="J137" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K137" s="0" t="s">
+      <c r="K137" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L137" s="0" t="s">
+      <c r="L137" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7654,10 +7653,10 @@
       <c r="J138" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K138" s="0" t="s">
+      <c r="K138" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L138" s="0" t="s">
+      <c r="L138" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7689,10 +7688,10 @@
       <c r="J139" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K139" s="0" t="s">
+      <c r="K139" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L139" s="0" t="s">
+      <c r="L139" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7724,10 +7723,10 @@
       <c r="J140" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K140" s="0" t="s">
+      <c r="K140" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L140" s="0" t="s">
+      <c r="L140" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7759,10 +7758,10 @@
       <c r="J141" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K141" s="0" t="s">
+      <c r="K141" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L141" s="0" t="s">
+      <c r="L141" s="1" t="s">
         <v>150</v>
       </c>
     </row>
@@ -7794,10 +7793,10 @@
       <c r="J142" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K142" s="0" t="s">
+      <c r="K142" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L142" s="0" t="s">
+      <c r="L142" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -7829,10 +7828,10 @@
       <c r="J143" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K143" s="0" t="s">
+      <c r="K143" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L143" s="0" t="s">
+      <c r="L143" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -7864,10 +7863,10 @@
       <c r="J144" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K144" s="0" t="s">
+      <c r="K144" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L144" s="0" t="s">
+      <c r="L144" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -7899,10 +7898,10 @@
       <c r="J145" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K145" s="0" t="s">
+      <c r="K145" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L145" s="0" t="s">
+      <c r="L145" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -7934,10 +7933,10 @@
       <c r="J146" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K146" s="0" t="s">
+      <c r="K146" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L146" s="0" t="s">
+      <c r="L146" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -7969,10 +7968,10 @@
       <c r="J147" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K147" s="0" t="s">
+      <c r="K147" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L147" s="0" t="s">
+      <c r="L147" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -8004,10 +8003,10 @@
       <c r="J148" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K148" s="0" t="s">
+      <c r="K148" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L148" s="0" t="s">
+      <c r="L148" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -8039,10 +8038,10 @@
       <c r="J149" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K149" s="0" t="s">
+      <c r="K149" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L149" s="0" t="s">
+      <c r="L149" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -8074,10 +8073,10 @@
       <c r="J150" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K150" s="0" t="s">
+      <c r="K150" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L150" s="0" t="s">
+      <c r="L150" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -8109,10 +8108,10 @@
       <c r="J151" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="K151" s="0" t="s">
+      <c r="K151" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="L151" s="0" t="s">
+      <c r="L151" s="1" t="s">
         <v>116</v>
       </c>
     </row>
@@ -8144,10 +8143,10 @@
       <c r="J152" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K152" s="0" t="s">
+      <c r="K152" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L152" s="0" t="s">
+      <c r="L152" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8179,10 +8178,10 @@
       <c r="J153" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K153" s="0" t="s">
+      <c r="K153" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L153" s="0" t="s">
+      <c r="L153" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8214,10 +8213,10 @@
       <c r="J154" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K154" s="0" t="s">
+      <c r="K154" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L154" s="0" t="s">
+      <c r="L154" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8249,10 +8248,10 @@
       <c r="J155" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K155" s="0" t="s">
+      <c r="K155" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L155" s="0" t="s">
+      <c r="L155" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8284,10 +8283,10 @@
       <c r="J156" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K156" s="0" t="s">
+      <c r="K156" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L156" s="0" t="s">
+      <c r="L156" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8319,10 +8318,10 @@
       <c r="J157" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K157" s="0" t="s">
+      <c r="K157" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L157" s="0" t="s">
+      <c r="L157" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8354,10 +8353,10 @@
       <c r="J158" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K158" s="0" t="s">
+      <c r="K158" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L158" s="0" t="s">
+      <c r="L158" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8389,10 +8388,10 @@
       <c r="J159" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K159" s="0" t="s">
+      <c r="K159" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L159" s="0" t="s">
+      <c r="L159" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8424,10 +8423,10 @@
       <c r="J160" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K160" s="0" t="s">
+      <c r="K160" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L160" s="0" t="s">
+      <c r="L160" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8459,10 +8458,10 @@
       <c r="J161" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="K161" s="0" t="s">
+      <c r="K161" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="L161" s="0" t="s">
+      <c r="L161" s="1" t="s">
         <v>138</v>
       </c>
     </row>
@@ -8494,10 +8493,10 @@
       <c r="J162" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K162" s="0" t="s">
+      <c r="K162" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L162" s="0" t="s">
+      <c r="L162" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8529,10 +8528,10 @@
       <c r="J163" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K163" s="0" t="s">
+      <c r="K163" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L163" s="0" t="s">
+      <c r="L163" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8564,10 +8563,10 @@
       <c r="J164" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K164" s="0" t="s">
+      <c r="K164" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L164" s="0" t="s">
+      <c r="L164" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8599,10 +8598,10 @@
       <c r="J165" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K165" s="0" t="s">
+      <c r="K165" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L165" s="0" t="s">
+      <c r="L165" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8634,10 +8633,10 @@
       <c r="J166" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K166" s="0" t="s">
+      <c r="K166" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L166" s="0" t="s">
+      <c r="L166" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8669,10 +8668,10 @@
       <c r="J167" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K167" s="0" t="s">
+      <c r="K167" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L167" s="0" t="s">
+      <c r="L167" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8704,10 +8703,10 @@
       <c r="J168" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K168" s="0" t="s">
+      <c r="K168" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L168" s="0" t="s">
+      <c r="L168" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8739,10 +8738,10 @@
       <c r="J169" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K169" s="0" t="s">
+      <c r="K169" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L169" s="0" t="s">
+      <c r="L169" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8774,10 +8773,10 @@
       <c r="J170" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K170" s="0" t="s">
+      <c r="K170" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L170" s="0" t="s">
+      <c r="L170" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8809,10 +8808,10 @@
       <c r="J171" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="K171" s="0" t="s">
+      <c r="K171" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L171" s="0" t="s">
+      <c r="L171" s="1" t="s">
         <v>163</v>
       </c>
     </row>
@@ -8844,10 +8843,10 @@
       <c r="J172" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K172" s="0" t="s">
+      <c r="K172" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L172" s="0" t="s">
+      <c r="L172" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -8879,10 +8878,10 @@
       <c r="J173" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K173" s="0" t="s">
+      <c r="K173" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L173" s="0" t="s">
+      <c r="L173" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -8914,10 +8913,10 @@
       <c r="J174" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K174" s="0" t="s">
+      <c r="K174" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L174" s="0" t="s">
+      <c r="L174" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -8949,10 +8948,10 @@
       <c r="J175" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K175" s="0" t="s">
+      <c r="K175" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L175" s="0" t="s">
+      <c r="L175" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -8984,7 +8983,7 @@
       <c r="J176" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K176" s="0" t="s">
+      <c r="K176" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -9016,10 +9015,10 @@
       <c r="J177" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K177" s="0" t="s">
+      <c r="K177" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L177" s="0" t="s">
+      <c r="L177" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9051,10 +9050,10 @@
       <c r="J178" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K178" s="0" t="s">
+      <c r="K178" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L178" s="0" t="s">
+      <c r="L178" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9086,10 +9085,10 @@
       <c r="J179" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K179" s="0" t="s">
+      <c r="K179" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L179" s="0" t="s">
+      <c r="L179" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9121,10 +9120,10 @@
       <c r="J180" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K180" s="0" t="s">
+      <c r="K180" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L180" s="0" t="s">
+      <c r="L180" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9156,10 +9155,10 @@
       <c r="J181" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K181" s="0" t="s">
+      <c r="K181" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L181" s="0" t="s">
+      <c r="L181" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9191,7 +9190,7 @@
       <c r="J182" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K182" s="0" t="s">
+      <c r="K182" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -9223,10 +9222,10 @@
       <c r="J183" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K183" s="0" t="s">
+      <c r="K183" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L183" s="0" t="s">
+      <c r="L183" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9258,10 +9257,10 @@
       <c r="J184" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K184" s="0" t="s">
+      <c r="K184" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L184" s="0" t="s">
+      <c r="L184" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9293,7 +9292,7 @@
       <c r="J185" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K185" s="0" t="s">
+      <c r="K185" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -9325,10 +9324,10 @@
       <c r="J186" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K186" s="0" t="s">
+      <c r="K186" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L186" s="0" t="s">
+      <c r="L186" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -9360,7 +9359,7 @@
       <c r="J187" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K187" s="0" t="s">
+      <c r="K187" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -9392,10 +9391,10 @@
       <c r="J188" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K188" s="0" t="s">
+      <c r="K188" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L188" s="0" t="s">
+      <c r="L188" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9427,10 +9426,10 @@
       <c r="J189" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K189" s="0" t="s">
+      <c r="K189" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L189" s="0" t="s">
+      <c r="L189" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9462,10 +9461,10 @@
       <c r="J190" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K190" s="0" t="s">
+      <c r="K190" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L190" s="0" t="s">
+      <c r="L190" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9497,7 +9496,7 @@
       <c r="J191" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K191" s="0" t="s">
+      <c r="K191" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -9529,10 +9528,10 @@
       <c r="J192" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K192" s="0" t="s">
+      <c r="K192" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L192" s="0" t="s">
+      <c r="L192" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9564,10 +9563,10 @@
       <c r="J193" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K193" s="0" t="s">
+      <c r="K193" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L193" s="0" t="s">
+      <c r="L193" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9599,10 +9598,10 @@
       <c r="J194" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K194" s="0" t="s">
+      <c r="K194" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L194" s="0" t="s">
+      <c r="L194" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9634,7 +9633,7 @@
       <c r="J195" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K195" s="0" t="s">
+      <c r="K195" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -9666,7 +9665,7 @@
       <c r="J196" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K196" s="0" t="s">
+      <c r="K196" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -9698,10 +9697,10 @@
       <c r="J197" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K197" s="0" t="s">
+      <c r="K197" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L197" s="0" t="s">
+      <c r="L197" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9733,10 +9732,10 @@
       <c r="J198" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K198" s="0" t="s">
+      <c r="K198" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L198" s="0" t="s">
+      <c r="L198" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9768,10 +9767,10 @@
       <c r="J199" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K199" s="0" t="s">
+      <c r="K199" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L199" s="0" t="s">
+      <c r="L199" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9803,10 +9802,10 @@
       <c r="J200" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K200" s="0" t="s">
+      <c r="K200" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L200" s="0" t="s">
+      <c r="L200" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -9838,10 +9837,10 @@
       <c r="J201" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K201" s="0" t="s">
+      <c r="K201" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L201" s="0" t="s">
+      <c r="L201" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -9873,10 +9872,10 @@
       <c r="J202" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K202" s="0" t="s">
+      <c r="K202" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L202" s="0" t="s">
+      <c r="L202" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -9908,7 +9907,7 @@
       <c r="J203" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K203" s="0" t="s">
+      <c r="K203" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -9940,10 +9939,10 @@
       <c r="J204" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K204" s="0" t="s">
+      <c r="K204" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L204" s="0" t="s">
+      <c r="L204" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -9975,10 +9974,10 @@
       <c r="J205" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K205" s="0" t="s">
+      <c r="K205" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L205" s="0" t="s">
+      <c r="L205" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10010,7 +10009,7 @@
       <c r="J206" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K206" s="0" t="s">
+      <c r="K206" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -10042,7 +10041,7 @@
       <c r="J207" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K207" s="0" t="s">
+      <c r="K207" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -10074,10 +10073,10 @@
       <c r="J208" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K208" s="0" t="s">
+      <c r="K208" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L208" s="0" t="s">
+      <c r="L208" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10109,10 +10108,10 @@
       <c r="J209" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K209" s="0" t="s">
+      <c r="K209" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L209" s="0" t="s">
+      <c r="L209" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10144,10 +10143,10 @@
       <c r="J210" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K210" s="0" t="s">
+      <c r="K210" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L210" s="0" t="s">
+      <c r="L210" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10179,10 +10178,10 @@
       <c r="J211" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K211" s="0" t="s">
+      <c r="K211" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L211" s="0" t="s">
+      <c r="L211" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10214,10 +10213,10 @@
       <c r="J212" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K212" s="0" t="s">
+      <c r="K212" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L212" s="0" t="s">
+      <c r="L212" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10249,10 +10248,10 @@
       <c r="J213" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K213" s="0" t="s">
+      <c r="K213" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L213" s="0" t="s">
+      <c r="L213" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10284,10 +10283,10 @@
       <c r="J214" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K214" s="0" t="s">
+      <c r="K214" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L214" s="0" t="s">
+      <c r="L214" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -10319,7 +10318,7 @@
       <c r="J215" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K215" s="0" t="s">
+      <c r="K215" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -10351,10 +10350,10 @@
       <c r="J216" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K216" s="0" t="s">
+      <c r="K216" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L216" s="0" t="s">
+      <c r="L216" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -10386,10 +10385,10 @@
       <c r="J217" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K217" s="0" t="s">
+      <c r="K217" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L217" s="0" t="s">
+      <c r="L217" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -10421,10 +10420,10 @@
       <c r="J218" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K218" s="0" t="s">
+      <c r="K218" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L218" s="0" t="s">
+      <c r="L218" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -10456,10 +10455,10 @@
       <c r="J219" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K219" s="0" t="s">
+      <c r="K219" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L219" s="0" t="s">
+      <c r="L219" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10491,10 +10490,10 @@
       <c r="J220" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K220" s="0" t="s">
+      <c r="K220" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L220" s="0" t="s">
+      <c r="L220" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10526,10 +10525,10 @@
       <c r="J221" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K221" s="0" t="s">
+      <c r="K221" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L221" s="0" t="s">
+      <c r="L221" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10561,10 +10560,10 @@
       <c r="J222" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K222" s="0" t="s">
+      <c r="K222" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L222" s="0" t="s">
+      <c r="L222" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10596,10 +10595,10 @@
       <c r="J223" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K223" s="0" t="s">
+      <c r="K223" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L223" s="0" t="s">
+      <c r="L223" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10631,10 +10630,10 @@
       <c r="J224" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K224" s="0" t="s">
+      <c r="K224" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L224" s="0" t="s">
+      <c r="L224" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10666,10 +10665,10 @@
       <c r="J225" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K225" s="0" t="s">
+      <c r="K225" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L225" s="0" t="s">
+      <c r="L225" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10701,10 +10700,10 @@
       <c r="J226" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K226" s="0" t="s">
+      <c r="K226" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L226" s="0" t="s">
+      <c r="L226" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10736,10 +10735,10 @@
       <c r="J227" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K227" s="0" t="s">
+      <c r="K227" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="L227" s="0" t="s">
+      <c r="L227" s="1" t="s">
         <v>231</v>
       </c>
     </row>
@@ -10771,10 +10770,10 @@
       <c r="J228" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K228" s="0" t="s">
+      <c r="K228" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L228" s="0" t="s">
+      <c r="L228" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10806,10 +10805,10 @@
       <c r="J229" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K229" s="0" t="s">
+      <c r="K229" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L229" s="0" t="s">
+      <c r="L229" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10841,10 +10840,10 @@
       <c r="J230" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K230" s="0" t="s">
+      <c r="K230" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L230" s="0" t="s">
+      <c r="L230" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -10876,10 +10875,10 @@
       <c r="J231" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K231" s="0" t="s">
+      <c r="K231" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L231" s="0" t="s">
+      <c r="L231" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -10911,10 +10910,10 @@
       <c r="J232" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K232" s="0" t="s">
+      <c r="K232" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L232" s="0" t="s">
+      <c r="L232" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -10946,10 +10945,10 @@
       <c r="J233" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K233" s="0" t="s">
+      <c r="K233" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L233" s="0" t="s">
+      <c r="L233" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -10981,10 +10980,10 @@
       <c r="J234" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K234" s="0" t="s">
+      <c r="K234" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L234" s="0" t="s">
+      <c r="L234" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -11016,10 +11015,10 @@
       <c r="J235" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K235" s="0" t="s">
+      <c r="K235" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L235" s="0" t="s">
+      <c r="L235" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11051,10 +11050,10 @@
       <c r="J236" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K236" s="0" t="s">
+      <c r="K236" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L236" s="0" t="s">
+      <c r="L236" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11086,10 +11085,10 @@
       <c r="J237" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K237" s="0" t="s">
+      <c r="K237" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L237" s="0" t="s">
+      <c r="L237" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11121,10 +11120,10 @@
       <c r="J238" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K238" s="0" t="s">
+      <c r="K238" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L238" s="0" t="s">
+      <c r="L238" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -11156,7 +11155,7 @@
       <c r="J239" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K239" s="0" t="s">
+      <c r="K239" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -11188,10 +11187,10 @@
       <c r="J240" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K240" s="0" t="s">
+      <c r="K240" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L240" s="0" t="s">
+      <c r="L240" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11223,10 +11222,10 @@
       <c r="J241" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K241" s="0" t="s">
+      <c r="K241" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L241" s="0" t="s">
+      <c r="L241" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11258,10 +11257,10 @@
       <c r="J242" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K242" s="0" t="s">
+      <c r="K242" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L242" s="0" t="s">
+      <c r="L242" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11293,10 +11292,10 @@
       <c r="J243" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K243" s="0" t="s">
+      <c r="K243" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L243" s="0" t="s">
+      <c r="L243" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11328,10 +11327,10 @@
       <c r="J244" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K244" s="0" t="s">
+      <c r="K244" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L244" s="0" t="s">
+      <c r="L244" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11363,10 +11362,10 @@
       <c r="J245" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K245" s="0" t="s">
+      <c r="K245" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L245" s="0" t="s">
+      <c r="L245" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -11398,10 +11397,10 @@
       <c r="J246" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K246" s="0" t="s">
+      <c r="K246" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L246" s="0" t="s">
+      <c r="L246" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11433,10 +11432,10 @@
       <c r="J247" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K247" s="0" t="s">
+      <c r="K247" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L247" s="0" t="s">
+      <c r="L247" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -11468,10 +11467,10 @@
       <c r="J248" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K248" s="0" t="s">
+      <c r="K248" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L248" s="0" t="s">
+      <c r="L248" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11503,10 +11502,10 @@
       <c r="J249" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K249" s="0" t="s">
+      <c r="K249" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L249" s="0" t="s">
+      <c r="L249" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11538,10 +11537,10 @@
       <c r="J250" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K250" s="0" t="s">
+      <c r="K250" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L250" s="0" t="s">
+      <c r="L250" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11573,10 +11572,10 @@
       <c r="J251" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K251" s="0" t="s">
+      <c r="K251" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L251" s="0" t="s">
+      <c r="L251" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -11608,10 +11607,10 @@
       <c r="J252" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K252" s="0" t="s">
+      <c r="K252" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L252" s="0" t="s">
+      <c r="L252" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11643,10 +11642,10 @@
       <c r="J253" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K253" s="0" t="s">
+      <c r="K253" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L253" s="0" t="s">
+      <c r="L253" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -11678,7 +11677,7 @@
       <c r="J254" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K254" s="0" t="s">
+      <c r="K254" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -11710,10 +11709,10 @@
       <c r="J255" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K255" s="0" t="s">
+      <c r="K255" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L255" s="0" t="s">
+      <c r="L255" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11745,10 +11744,10 @@
       <c r="J256" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K256" s="0" t="s">
+      <c r="K256" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L256" s="0" t="s">
+      <c r="L256" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -11780,7 +11779,7 @@
       <c r="J257" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K257" s="0" t="s">
+      <c r="K257" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -11812,10 +11811,10 @@
       <c r="J258" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K258" s="0" t="s">
+      <c r="K258" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L258" s="0" t="s">
+      <c r="L258" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11847,10 +11846,10 @@
       <c r="J259" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K259" s="0" t="s">
+      <c r="K259" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L259" s="0" t="s">
+      <c r="L259" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11882,10 +11881,10 @@
       <c r="J260" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K260" s="0" t="s">
+      <c r="K260" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L260" s="0" t="s">
+      <c r="L260" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -11917,10 +11916,10 @@
       <c r="J261" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K261" s="0" t="s">
+      <c r="K261" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L261" s="0" t="s">
+      <c r="L261" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -11952,10 +11951,10 @@
       <c r="J262" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K262" s="0" t="s">
+      <c r="K262" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L262" s="0" t="s">
+      <c r="L262" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -11987,10 +11986,10 @@
       <c r="J263" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K263" s="0" t="s">
+      <c r="K263" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L263" s="0" t="s">
+      <c r="L263" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12022,10 +12021,10 @@
       <c r="J264" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K264" s="0" t="s">
+      <c r="K264" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L264" s="0" t="s">
+      <c r="L264" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -12057,10 +12056,10 @@
       <c r="J265" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K265" s="0" t="s">
+      <c r="K265" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L265" s="0" t="s">
+      <c r="L265" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12092,10 +12091,10 @@
       <c r="J266" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K266" s="0" t="s">
+      <c r="K266" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L266" s="0" t="s">
+      <c r="L266" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12127,10 +12126,10 @@
       <c r="J267" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K267" s="0" t="s">
+      <c r="K267" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L267" s="0" t="s">
+      <c r="L267" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -12162,10 +12161,10 @@
       <c r="J268" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K268" s="0" t="s">
+      <c r="K268" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L268" s="0" t="s">
+      <c r="L268" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12197,10 +12196,10 @@
       <c r="J269" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K269" s="0" t="s">
+      <c r="K269" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L269" s="0" t="s">
+      <c r="L269" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -12232,10 +12231,10 @@
       <c r="J270" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K270" s="0" t="s">
+      <c r="K270" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L270" s="0" t="s">
+      <c r="L270" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12267,10 +12266,10 @@
       <c r="J271" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K271" s="0" t="s">
+      <c r="K271" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L271" s="0" t="s">
+      <c r="L271" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -12302,10 +12301,10 @@
       <c r="J272" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K272" s="0" t="s">
+      <c r="K272" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L272" s="0" t="s">
+      <c r="L272" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12337,10 +12336,10 @@
       <c r="J273" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K273" s="0" t="s">
+      <c r="K273" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L273" s="0" t="s">
+      <c r="L273" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12372,10 +12371,10 @@
       <c r="J274" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K274" s="0" t="s">
+      <c r="K274" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L274" s="0" t="s">
+      <c r="L274" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -12407,10 +12406,10 @@
       <c r="J275" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="K275" s="0" t="s">
+      <c r="K275" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="L275" s="0" t="s">
+      <c r="L275" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -12442,10 +12441,10 @@
       <c r="J276" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K276" s="0" t="s">
+      <c r="K276" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L276" s="0" t="s">
+      <c r="L276" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12477,10 +12476,10 @@
       <c r="J277" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="K277" s="0" t="s">
+      <c r="K277" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L277" s="0" t="s">
+      <c r="L277" s="1" t="s">
         <v>285</v>
       </c>
     </row>
@@ -12512,10 +12511,10 @@
       <c r="J278" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K278" s="0" t="s">
+      <c r="K278" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L278" s="0" t="s">
+      <c r="L278" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -12547,10 +12546,10 @@
       <c r="J279" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K279" s="0" t="s">
+      <c r="K279" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L279" s="0" t="s">
+      <c r="L279" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12582,10 +12581,10 @@
       <c r="J280" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K280" s="0" t="s">
+      <c r="K280" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L280" s="0" t="s">
+      <c r="L280" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12617,10 +12616,10 @@
       <c r="J281" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K281" s="0" t="s">
+      <c r="K281" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L281" s="0" t="s">
+      <c r="L281" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12652,10 +12651,10 @@
       <c r="J282" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K282" s="0" t="s">
+      <c r="K282" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L282" s="0" t="s">
+      <c r="L282" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12687,10 +12686,10 @@
       <c r="J283" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K283" s="0" t="s">
+      <c r="K283" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L283" s="0" t="s">
+      <c r="L283" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12722,10 +12721,10 @@
       <c r="J284" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K284" s="0" t="s">
+      <c r="K284" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L284" s="0" t="s">
+      <c r="L284" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12757,10 +12756,10 @@
       <c r="J285" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K285" s="0" t="s">
+      <c r="K285" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L285" s="0" t="s">
+      <c r="L285" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12792,10 +12791,10 @@
       <c r="J286" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K286" s="0" t="s">
+      <c r="K286" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L286" s="0" t="s">
+      <c r="L286" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -12827,10 +12826,10 @@
       <c r="J287" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K287" s="0" t="s">
+      <c r="K287" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L287" s="0" t="s">
+      <c r="L287" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -12862,10 +12861,10 @@
       <c r="J288" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K288" s="0" t="s">
+      <c r="K288" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L288" s="0" t="s">
+      <c r="L288" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12897,10 +12896,10 @@
       <c r="J289" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K289" s="0" t="s">
+      <c r="K289" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L289" s="0" t="s">
+      <c r="L289" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12932,10 +12931,10 @@
       <c r="J290" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K290" s="0" t="s">
+      <c r="K290" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L290" s="0" t="s">
+      <c r="L290" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -12967,10 +12966,10 @@
       <c r="J291" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K291" s="0" t="s">
+      <c r="K291" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L291" s="0" t="s">
+      <c r="L291" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -13002,10 +13001,10 @@
       <c r="J292" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K292" s="0" t="s">
+      <c r="K292" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L292" s="0" t="s">
+      <c r="L292" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13037,10 +13036,10 @@
       <c r="J293" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K293" s="0" t="s">
+      <c r="K293" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L293" s="0" t="s">
+      <c r="L293" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13072,10 +13071,10 @@
       <c r="J294" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K294" s="0" t="s">
+      <c r="K294" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L294" s="0" t="s">
+      <c r="L294" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13107,10 +13106,10 @@
       <c r="J295" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K295" s="0" t="s">
+      <c r="K295" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L295" s="0" t="s">
+      <c r="L295" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13142,10 +13141,10 @@
       <c r="J296" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K296" s="0" t="s">
+      <c r="K296" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L296" s="0" t="s">
+      <c r="L296" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13177,10 +13176,10 @@
       <c r="J297" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K297" s="0" t="s">
+      <c r="K297" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L297" s="0" t="s">
+      <c r="L297" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13212,10 +13211,10 @@
       <c r="J298" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K298" s="0" t="s">
+      <c r="K298" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L298" s="0" t="s">
+      <c r="L298" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13247,10 +13246,10 @@
       <c r="J299" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K299" s="0" t="s">
+      <c r="K299" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L299" s="0" t="s">
+      <c r="L299" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13282,10 +13281,10 @@
       <c r="J300" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K300" s="0" t="s">
+      <c r="K300" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L300" s="0" t="s">
+      <c r="L300" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13317,10 +13316,10 @@
       <c r="J301" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K301" s="0" t="s">
+      <c r="K301" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L301" s="0" t="s">
+      <c r="L301" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13352,10 +13351,10 @@
       <c r="J302" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K302" s="0" t="s">
+      <c r="K302" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L302" s="0" t="s">
+      <c r="L302" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13387,10 +13386,10 @@
       <c r="J303" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K303" s="0" t="s">
+      <c r="K303" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L303" s="0" t="s">
+      <c r="L303" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13422,10 +13421,10 @@
       <c r="J304" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K304" s="0" t="s">
+      <c r="K304" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L304" s="0" t="s">
+      <c r="L304" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -13457,10 +13456,10 @@
       <c r="J305" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K305" s="0" t="s">
+      <c r="K305" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L305" s="0" t="s">
+      <c r="L305" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -13492,10 +13491,10 @@
       <c r="J306" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="K306" s="0" t="s">
+      <c r="K306" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L306" s="0" t="s">
+      <c r="L306" s="1" t="s">
         <v>327</v>
       </c>
     </row>
@@ -13527,10 +13526,10 @@
       <c r="J307" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K307" s="0" t="s">
+      <c r="K307" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L307" s="0" t="s">
+      <c r="L307" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13562,10 +13561,10 @@
       <c r="J308" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K308" s="0" t="s">
+      <c r="K308" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L308" s="0" t="s">
+      <c r="L308" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13597,10 +13596,10 @@
       <c r="J309" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K309" s="0" t="s">
+      <c r="K309" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L309" s="0" t="s">
+      <c r="L309" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13632,10 +13631,10 @@
       <c r="J310" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K310" s="0" t="s">
+      <c r="K310" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L310" s="0" t="s">
+      <c r="L310" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13667,10 +13666,10 @@
       <c r="J311" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K311" s="0" t="s">
+      <c r="K311" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L311" s="0" t="s">
+      <c r="L311" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13702,10 +13701,10 @@
       <c r="J312" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K312" s="0" t="s">
+      <c r="K312" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L312" s="0" t="s">
+      <c r="L312" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13737,10 +13736,10 @@
       <c r="J313" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K313" s="0" t="s">
+      <c r="K313" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L313" s="0" t="s">
+      <c r="L313" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13772,10 +13771,10 @@
       <c r="J314" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K314" s="0" t="s">
+      <c r="K314" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L314" s="0" t="s">
+      <c r="L314" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13807,10 +13806,10 @@
       <c r="J315" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K315" s="0" t="s">
+      <c r="K315" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L315" s="0" t="s">
+      <c r="L315" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13842,10 +13841,10 @@
       <c r="J316" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K316" s="0" t="s">
+      <c r="K316" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L316" s="0" t="s">
+      <c r="L316" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13877,10 +13876,10 @@
       <c r="J317" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K317" s="0" t="s">
+      <c r="K317" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L317" s="0" t="s">
+      <c r="L317" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13912,10 +13911,10 @@
       <c r="J318" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K318" s="0" t="s">
+      <c r="K318" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L318" s="0" t="s">
+      <c r="L318" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13947,10 +13946,10 @@
       <c r="J319" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K319" s="0" t="s">
+      <c r="K319" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L319" s="0" t="s">
+      <c r="L319" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -13982,10 +13981,10 @@
       <c r="J320" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K320" s="0" t="s">
+      <c r="K320" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L320" s="0" t="s">
+      <c r="L320" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -14017,10 +14016,10 @@
       <c r="J321" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="K321" s="0" t="s">
+      <c r="K321" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L321" s="0" t="s">
+      <c r="L321" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -14052,10 +14051,10 @@
       <c r="J322" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="K322" s="0" t="s">
+      <c r="K322" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L322" s="0" t="s">
+      <c r="L322" s="1" t="s">
         <v>285</v>
       </c>
     </row>
@@ -14087,10 +14086,10 @@
       <c r="J323" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="K323" s="0" t="s">
+      <c r="K323" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L323" s="0" t="s">
+      <c r="L323" s="1" t="s">
         <v>285</v>
       </c>
     </row>
@@ -14122,10 +14121,10 @@
       <c r="J324" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K324" s="0" t="s">
+      <c r="K324" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L324" s="0" t="s">
+      <c r="L324" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14157,10 +14156,10 @@
       <c r="J325" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="K325" s="0" t="s">
+      <c r="K325" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L325" s="0" t="s">
+      <c r="L325" s="1" t="s">
         <v>285</v>
       </c>
     </row>
@@ -14192,10 +14191,10 @@
       <c r="J326" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K326" s="0" t="s">
+      <c r="K326" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L326" s="0" t="s">
+      <c r="L326" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14227,10 +14226,10 @@
       <c r="J327" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K327" s="0" t="s">
+      <c r="K327" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L327" s="0" t="s">
+      <c r="L327" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14262,10 +14261,10 @@
       <c r="J328" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K328" s="0" t="s">
+      <c r="K328" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L328" s="0" t="s">
+      <c r="L328" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14297,10 +14296,10 @@
       <c r="J329" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K329" s="0" t="s">
+      <c r="K329" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L329" s="0" t="s">
+      <c r="L329" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14332,10 +14331,10 @@
       <c r="J330" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K330" s="0" t="s">
+      <c r="K330" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L330" s="0" t="s">
+      <c r="L330" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -14367,10 +14366,10 @@
       <c r="J331" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="K331" s="0" t="s">
+      <c r="K331" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="L331" s="0" t="s">
+      <c r="L331" s="1" t="s">
         <v>280</v>
       </c>
     </row>
@@ -14402,10 +14401,10 @@
       <c r="J332" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="K332" s="0" t="s">
+      <c r="K332" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L332" s="0" t="s">
+      <c r="L332" s="1" t="s">
         <v>285</v>
       </c>
     </row>
@@ -14437,10 +14436,10 @@
       <c r="J333" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K333" s="0" t="s">
+      <c r="K333" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L333" s="0" t="s">
+      <c r="L333" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14472,10 +14471,10 @@
       <c r="J334" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K334" s="0" t="s">
+      <c r="K334" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L334" s="0" t="s">
+      <c r="L334" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14507,10 +14506,10 @@
       <c r="J335" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="K335" s="0" t="s">
+      <c r="K335" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="L335" s="0" t="s">
+      <c r="L335" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -14542,10 +14541,10 @@
       <c r="J336" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="K336" s="0" t="s">
+      <c r="K336" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L336" s="0" t="s">
+      <c r="L336" s="1" t="s">
         <v>327</v>
       </c>
     </row>
@@ -14577,10 +14576,10 @@
       <c r="J337" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K337" s="0" t="s">
+      <c r="K337" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L337" s="0" t="s">
+      <c r="L337" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -14612,10 +14611,10 @@
       <c r="J338" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K338" s="0" t="s">
+      <c r="K338" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L338" s="0" t="s">
+      <c r="L338" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -14647,10 +14646,10 @@
       <c r="J339" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K339" s="0" t="s">
+      <c r="K339" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L339" s="0" t="s">
+      <c r="L339" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -14682,10 +14681,10 @@
       <c r="J340" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="K340" s="0" t="s">
+      <c r="K340" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L340" s="0" t="s">
+      <c r="L340" s="1" t="s">
         <v>327</v>
       </c>
     </row>
@@ -14717,10 +14716,10 @@
       <c r="J341" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="K341" s="0" t="s">
+      <c r="K341" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L341" s="0" t="s">
+      <c r="L341" s="1" t="s">
         <v>327</v>
       </c>
     </row>
@@ -14752,10 +14751,10 @@
       <c r="J342" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K342" s="0" t="s">
+      <c r="K342" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L342" s="0" t="s">
+      <c r="L342" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -14787,10 +14786,10 @@
       <c r="J343" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K343" s="0" t="s">
+      <c r="K343" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L343" s="0" t="s">
+      <c r="L343" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -14822,10 +14821,10 @@
       <c r="J344" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="K344" s="0" t="s">
+      <c r="K344" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="L344" s="0" t="s">
+      <c r="L344" s="1" t="s">
         <v>327</v>
       </c>
     </row>
@@ -14857,10 +14856,10 @@
       <c r="J345" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K345" s="0" t="s">
+      <c r="K345" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L345" s="0" t="s">
+      <c r="L345" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -14892,10 +14891,10 @@
       <c r="J346" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K346" s="0" t="s">
+      <c r="K346" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L346" s="0" t="s">
+      <c r="L346" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -14927,10 +14926,10 @@
       <c r="J347" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K347" s="0" t="s">
+      <c r="K347" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L347" s="0" t="s">
+      <c r="L347" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -14962,10 +14961,10 @@
       <c r="J348" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="K348" s="0" t="s">
+      <c r="K348" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="L348" s="0" t="s">
+      <c r="L348" s="1" t="s">
         <v>328</v>
       </c>
     </row>
@@ -14997,10 +14996,10 @@
       <c r="J349" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K349" s="0" t="s">
+      <c r="K349" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L349" s="0" t="s">
+      <c r="L349" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -15032,10 +15031,10 @@
       <c r="J350" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="K350" s="0" t="s">
+      <c r="K350" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="L350" s="0" t="s">
+      <c r="L350" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -15067,7 +15066,7 @@
       <c r="J351" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K351" s="0" t="s">
+      <c r="K351" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -15099,7 +15098,7 @@
       <c r="J352" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K352" s="0" t="s">
+      <c r="K352" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -15131,7 +15130,7 @@
       <c r="J353" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K353" s="0" t="s">
+      <c r="K353" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -15163,7 +15162,7 @@
       <c r="J354" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K354" s="0" t="s">
+      <c r="K354" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -15195,7 +15194,7 @@
       <c r="J355" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="K355" s="0" t="s">
+      <c r="K355" s="1" t="s">
         <v>281</v>
       </c>
     </row>
@@ -15227,7 +15226,7 @@
       <c r="J356" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K356" s="0" t="s">
+      <c r="K356" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15259,7 +15258,7 @@
       <c r="J357" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K357" s="0" t="s">
+      <c r="K357" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15291,7 +15290,7 @@
       <c r="J358" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K358" s="0" t="s">
+      <c r="K358" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15323,7 +15322,7 @@
       <c r="J359" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K359" s="0" t="s">
+      <c r="K359" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15355,7 +15354,7 @@
       <c r="J360" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K360" s="0" t="s">
+      <c r="K360" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15387,7 +15386,7 @@
       <c r="J361" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K361" s="0" t="s">
+      <c r="K361" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15419,7 +15418,7 @@
       <c r="J362" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K362" s="0" t="s">
+      <c r="K362" s="1" t="s">
         <v>229</v>
       </c>
     </row>
@@ -15451,7 +15450,7 @@
       <c r="J363" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K363" s="0" t="s">
+      <c r="K363" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -15483,7 +15482,7 @@
       <c r="J364" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K364" s="0" t="s">
+      <c r="K364" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -15515,7 +15514,7 @@
       <c r="J365" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K365" s="0" t="s">
+      <c r="K365" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -15547,7 +15546,7 @@
       <c r="J366" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="K366" s="0" t="s">
+      <c r="K366" s="1" t="s">
         <v>326</v>
       </c>
     </row>

</xml_diff>